<commit_message>
pre-release cleanup and master product support
</commit_message>
<xml_diff>
--- a/docs/批量更新库存.xlsx
+++ b/docs/批量更新库存.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\zhanghan\01-IT\03-soft\002-WMS\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CD4FF15-C830-4553-B3CA-42AE8AD37599}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A12E460-E671-4091-9387-EAA685D6ABFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-93" yWindow="-93" windowWidth="19386" windowHeight="12266" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,27 +27,15 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
   <si>
-    <r>
-      <t>SKU(fba</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Microsoft YaHei"/>
-        <family val="2"/>
-        <charset val="134"/>
-      </rPr>
-      <t>编码)</t>
-    </r>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>数量</t>
     <phoneticPr fontId="1"/>
   </si>
   <si>
     <t>箱号</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>产品ID</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -416,13 +404,13 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="C1" s="4" t="s">
         <v>0</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>1</v>
       </c>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>

</xml_diff>